<commit_message>
Corrí el script anterior sin dividir las especies por la distancia de dispersión
</commit_message>
<xml_diff>
--- a/resultados/ConR/criterioB/resumen_parametros_ConR.xlsx
+++ b/resultados/ConR/criterioB/resumen_parametros_ConR.xlsx
@@ -409,7 +409,7 @@
         <v>336</v>
       </c>
       <c r="F2">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H2">
         <v>56</v>
@@ -431,7 +431,7 @@
         <v>4</v>
       </c>
       <c r="H3">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -488,7 +488,7 @@
         <v>2</v>
       </c>
       <c r="H6">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -539,10 +539,10 @@
         <v>178347</v>
       </c>
       <c r="D9">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="F9">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H9">
         <v>28</v>
@@ -580,7 +580,7 @@
         <v>116</v>
       </c>
       <c r="F11">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H11">
         <v>19</v>
@@ -637,7 +637,7 @@
         <v>568</v>
       </c>
       <c r="F14">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H14">
         <v>89</v>
@@ -691,7 +691,7 @@
         <v>150772</v>
       </c>
       <c r="D17">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="F17">
         <v>20</v>
@@ -710,13 +710,13 @@
         <v>29789.9</v>
       </c>
       <c r="D18">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="F18">
         <v>5</v>
       </c>
       <c r="H18">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19">
@@ -770,7 +770,7 @@
         <v>28</v>
       </c>
       <c r="F21">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H21">
         <v>5</v>
@@ -808,7 +808,7 @@
         <v>156</v>
       </c>
       <c r="F23">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H23">
         <v>28</v>
@@ -849,7 +849,7 @@
         <v>1</v>
       </c>
       <c r="H25">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -865,7 +865,7 @@
         <v>360</v>
       </c>
       <c r="F26">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H26">
         <v>76</v>

</xml_diff>

<commit_message>
corrí el script con dispersión de 10 km
</commit_message>
<xml_diff>
--- a/resultados/ConR/criterioB/resumen_parametros_ConR.xlsx
+++ b/resultados/ConR/criterioB/resumen_parametros_ConR.xlsx
@@ -406,7 +406,7 @@
         <v>216517</v>
       </c>
       <c r="D2">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="F2">
         <v>66</v>
@@ -425,7 +425,7 @@
         <v>2182.1</v>
       </c>
       <c r="D3">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="F3">
         <v>4</v>
@@ -466,7 +466,7 @@
         <v>20</v>
       </c>
       <c r="F5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H5">
         <v>5</v>
@@ -539,10 +539,10 @@
         <v>178347</v>
       </c>
       <c r="D9">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="F9">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H9">
         <v>28</v>
@@ -558,7 +558,7 @@
         <v>319959</v>
       </c>
       <c r="D10">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="F10">
         <v>90</v>
@@ -634,10 +634,10 @@
         <v>354288</v>
       </c>
       <c r="D14">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="F14">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H14">
         <v>89</v>
@@ -710,7 +710,7 @@
         <v>29789.9</v>
       </c>
       <c r="D18">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="F18">
         <v>5</v>
@@ -770,7 +770,7 @@
         <v>28</v>
       </c>
       <c r="F21">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H21">
         <v>5</v>
@@ -789,7 +789,7 @@
         <v>16</v>
       </c>
       <c r="F22">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H22">
         <v>4</v>
@@ -865,7 +865,7 @@
         <v>360</v>
       </c>
       <c r="F26">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H26">
         <v>76</v>

</xml_diff>

<commit_message>
distancia dispersión 1km, HH 30%
</commit_message>
<xml_diff>
--- a/resultados/ConR/criterioB/resumen_parametros_ConR.xlsx
+++ b/resultados/ConR/criterioB/resumen_parametros_ConR.xlsx
@@ -406,13 +406,13 @@
         <v>216517</v>
       </c>
       <c r="D2">
-        <v>332</v>
+        <v>340</v>
       </c>
       <c r="F2">
         <v>66</v>
       </c>
       <c r="H2">
-        <v>56</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3">
@@ -425,13 +425,13 @@
         <v>2182.1</v>
       </c>
       <c r="D3">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="F3">
         <v>4</v>
       </c>
       <c r="H3">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -466,7 +466,7 @@
         <v>20</v>
       </c>
       <c r="F5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H5">
         <v>5</v>
@@ -488,7 +488,7 @@
         <v>2</v>
       </c>
       <c r="H6">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -526,7 +526,7 @@
         <v>17</v>
       </c>
       <c r="H8">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9">
@@ -545,7 +545,7 @@
         <v>35</v>
       </c>
       <c r="H9">
-        <v>28</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10">
@@ -558,13 +558,13 @@
         <v>319959</v>
       </c>
       <c r="D10">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="F10">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H10">
-        <v>75</v>
+        <v>107</v>
       </c>
     </row>
     <row r="11">
@@ -580,10 +580,10 @@
         <v>116</v>
       </c>
       <c r="F11">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H11">
-        <v>19</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12">
@@ -602,7 +602,7 @@
         <v>10</v>
       </c>
       <c r="H12">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13">
@@ -621,7 +621,7 @@
         <v>28</v>
       </c>
       <c r="H13">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14">
@@ -637,10 +637,10 @@
         <v>572</v>
       </c>
       <c r="F14">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="H14">
-        <v>89</v>
+        <v>140</v>
       </c>
     </row>
     <row r="15">
@@ -678,7 +678,7 @@
         <v>12</v>
       </c>
       <c r="H16">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17">
@@ -697,7 +697,7 @@
         <v>20</v>
       </c>
       <c r="H17">
-        <v>18</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18">
@@ -716,7 +716,7 @@
         <v>5</v>
       </c>
       <c r="H18">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19">
@@ -754,7 +754,7 @@
         <v>17</v>
       </c>
       <c r="H20">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21">
@@ -773,7 +773,7 @@
         <v>6</v>
       </c>
       <c r="H21">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="22">
@@ -789,7 +789,7 @@
         <v>16</v>
       </c>
       <c r="F22">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H22">
         <v>4</v>
@@ -805,13 +805,13 @@
         <v>196810</v>
       </c>
       <c r="D23">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="F23">
         <v>33</v>
       </c>
       <c r="H23">
-        <v>28</v>
+        <v>39</v>
       </c>
     </row>
     <row r="24">
@@ -830,7 +830,7 @@
         <v>32</v>
       </c>
       <c r="H24">
-        <v>29</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25">
@@ -849,7 +849,7 @@
         <v>1</v>
       </c>
       <c r="H25">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26">
@@ -865,10 +865,10 @@
         <v>360</v>
       </c>
       <c r="F26">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H26">
-        <v>76</v>
+        <v>89</v>
       </c>
     </row>
     <row r="27">
@@ -887,7 +887,7 @@
         <v>6</v>
       </c>
       <c r="H27">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
nuevo intento con 1km, 30%
</commit_message>
<xml_diff>
--- a/resultados/ConR/criterioB/resumen_parametros_ConR.xlsx
+++ b/resultados/ConR/criterioB/resumen_parametros_ConR.xlsx
@@ -406,10 +406,10 @@
         <v>216517</v>
       </c>
       <c r="D2">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="F2">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H2">
         <v>79</v>
@@ -428,7 +428,7 @@
         <v>32</v>
       </c>
       <c r="F3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H3">
         <v>8</v>
@@ -542,7 +542,7 @@
         <v>184</v>
       </c>
       <c r="F9">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H9">
         <v>44</v>
@@ -561,7 +561,7 @@
         <v>444</v>
       </c>
       <c r="F10">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H10">
         <v>107</v>
@@ -580,7 +580,7 @@
         <v>116</v>
       </c>
       <c r="F11">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H11">
         <v>28</v>
@@ -637,7 +637,7 @@
         <v>572</v>
       </c>
       <c r="F14">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="H14">
         <v>140</v>
@@ -710,7 +710,7 @@
         <v>29789.9</v>
       </c>
       <c r="D18">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="F18">
         <v>5</v>
@@ -865,7 +865,7 @@
         <v>360</v>
       </c>
       <c r="F26">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H26">
         <v>89</v>

</xml_diff>

<commit_message>
corrí por última vez todos los scripts con 1km, 30%
</commit_message>
<xml_diff>
--- a/resultados/ConR/criterioB/resumen_parametros_ConR.xlsx
+++ b/resultados/ConR/criterioB/resumen_parametros_ConR.xlsx
@@ -406,10 +406,10 @@
         <v>216517</v>
       </c>
       <c r="D2">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="F2">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H2">
         <v>79</v>
@@ -428,7 +428,7 @@
         <v>32</v>
       </c>
       <c r="F3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H3">
         <v>8</v>
@@ -539,7 +539,7 @@
         <v>178347</v>
       </c>
       <c r="D9">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="F9">
         <v>34</v>
@@ -558,7 +558,7 @@
         <v>319959</v>
       </c>
       <c r="D10">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="F10">
         <v>90</v>
@@ -637,7 +637,7 @@
         <v>572</v>
       </c>
       <c r="F14">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H14">
         <v>140</v>
@@ -710,7 +710,7 @@
         <v>29789.9</v>
       </c>
       <c r="D18">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="F18">
         <v>5</v>
@@ -770,7 +770,7 @@
         <v>28</v>
       </c>
       <c r="F21">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H21">
         <v>7</v>
@@ -827,7 +827,7 @@
         <v>152</v>
       </c>
       <c r="F24">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H24">
         <v>38</v>

</xml_diff>